<commit_message>
ajout datasheet + mise en forme git
</commit_message>
<xml_diff>
--- a/Banc de tests/mesures capteurs v1.xlsx
+++ b/Banc de tests/mesures capteurs v1.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/050671fe9a2caa0f/Documents/INSA/4A/Capteurs/2024-2025-4GP-Clara-Anatolie/Banc de tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B77437E2-7200-472B-8142-1DEDDEB09CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{B77437E2-7200-472B-8142-1DEDDEB09CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E291884B-2DD2-493C-A60D-628ED393D5BC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{EB6AD448-40F3-403B-81CE-D21654A49612}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{EB6AD448-40F3-403B-81CE-D21654A49612}"/>
   </bookViews>
   <sheets>
-    <sheet name="4B" sheetId="1" r:id="rId1"/>
-    <sheet name="5B" sheetId="2" r:id="rId2"/>
-    <sheet name="HB" sheetId="3" r:id="rId3"/>
+    <sheet name="4B tension" sheetId="1" r:id="rId1"/>
+    <sheet name="5B tension" sheetId="2" r:id="rId2"/>
+    <sheet name="HB tension" sheetId="3" r:id="rId3"/>
+    <sheet name="4B compr" sheetId="4" r:id="rId4"/>
+    <sheet name="5B compr" sheetId="5" r:id="rId5"/>
+    <sheet name="HB compr" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="10">
   <si>
     <t>|R|/R0</t>
   </si>
@@ -94,6 +97,12 @@
       <t>|/R0</t>
     </r>
   </si>
+  <si>
+    <t>R courbure</t>
+  </si>
+  <si>
+    <t>inf</t>
+  </si>
 </sst>
 </file>
 
@@ -120,12 +129,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -140,11 +155,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -201,7 +219,7 @@
             </a:r>
             <a:r>
               <a:rPr lang="fr-FR" baseline="0"/>
-              <a:t> change in resistance with respect to sensor deformation in relaxation</a:t>
+              <a:t> change in resistance with respect to sensor deformation in tension</a:t>
             </a:r>
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
@@ -294,34 +312,34 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'4B'!$B$3:$B$8</c:f>
+              <c:f>'4B tension'!$C$3:$C$8</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4.0000000000000001E-3</c:v>
+                  <c:v>2.1099999999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.1000000000000004E-3</c:v>
+                  <c:v>2.3800000000000002E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.3E-3</c:v>
+                  <c:v>2.7100000000000002E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.4999999999999997E-3</c:v>
+                  <c:v>3.1700000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.6999999999999994E-3</c:v>
+                  <c:v>3.8E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.01</c:v>
+                  <c:v>4.7499999999999999E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'4B'!$E$3:$E$8</c:f>
+              <c:f>'4B tension'!$F$3:$F$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -397,34 +415,34 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'5B'!$B$3:$B$8</c:f>
+              <c:f>'5B tension'!$C$3:$C$8</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4.0000000000000001E-3</c:v>
+                  <c:v>2.1099999999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.1000000000000004E-3</c:v>
+                  <c:v>2.3800000000000002E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.3E-3</c:v>
+                  <c:v>2.7100000000000002E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.4999999999999997E-3</c:v>
+                  <c:v>3.1700000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.6999999999999994E-3</c:v>
+                  <c:v>3.8E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.01</c:v>
+                  <c:v>4.7499999999999999E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'5B'!$E$3:$E$8</c:f>
+              <c:f>'5B tension'!$F$3:$F$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -500,28 +518,31 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>HB!$B$3:$B$6</c:f>
+              <c:f>'HB tension'!$C$3:$C$7</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.0000000000000001E-3</c:v>
+                  <c:v>2.1099999999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.3E-3</c:v>
+                  <c:v>2.7100000000000002E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.4999999999999997E-3</c:v>
+                  <c:v>3.1700000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.6999999999999994E-3</c:v>
+                  <c:v>3.8E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.7499999999999999E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>HB!$E$3:$E$7</c:f>
+              <c:f>'HB tension'!$F$3:$F$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -565,6 +586,7 @@
         <c:axId val="555954639"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="1.5000000000000005E-3"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -646,7 +668,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -969,31 +991,12 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'5B'!$B$3:$B$7</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>4.0000000000000001E-3</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5.1000000000000004E-3</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>6.3E-3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>7.4999999999999997E-3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>8.6999999999999994E-3</c:v>
-                </c:pt>
-              </c:numCache>
+              <c:f>'5B tension'!#REF!</c:f>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'5B'!$E$3:$E$7</c:f>
+              <c:f>'5B tension'!$F$3:$F$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -1264,7 +1267,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>HB!$E$1</c:f>
+              <c:f>'HB tension'!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1297,25 +1300,22 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>HB!$B$3:$B$5</c:f>
+              <c:f>'HB tension'!$C$3:$C$4</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>4.0000000000000001E-3</c:v>
+                  <c:v>2.1099999999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.3E-3</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>7.4999999999999997E-3</c:v>
+                  <c:v>2.7100000000000002E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>HB!$E$3:$E$6</c:f>
+              <c:f>'HB tension'!$F$3:$F$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1373,7 +1373,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1484,6 +1484,1551 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="fr-FR" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Relative change in resistance with respect to sensor deformation in compression</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.11143622805301399"/>
+          <c:y val="0.20912026332454603"/>
+          <c:w val="0.55107515776351168"/>
+          <c:h val="0.66091472950232744"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>4B Compression</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>('4B compr'!$C$3:$C$4,'4B compr'!$C$6:$C$7)</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2.1099999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.3800000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.1700000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.8E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>('4B compr'!$F$3:$F$4,'4B compr'!$F$6:$F$7)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>-1.1774877516571287E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-1.2515953723907942E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-2.4249660340071637E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-3.0116513648153487E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-CA89-4B9F-B6B5-36EEC4755D03}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>5B Compression</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'5B compr'!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2.1099999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.3800000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.7100000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.1700000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.8E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.7499999999999999E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'5B compr'!$F$3:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>-7.8586932115859588E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-1.0740214055834144E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-2.0657136441883092E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-2.7767382680937057E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-3.5008607140184118E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-4.9453633710051646E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-CA89-4B9F-B6B5-36EEC4755D03}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>HB Compression</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'HB compr'!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2.1099999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.3800000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.7100000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.1700000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.8E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.7499999999999999E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'HB compr'!$F$3:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>-1.641025641025641E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-3.2324786324786324E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-3.3490598290598292E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-3.433846153846154E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-4.0989743589743589E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-6.2745299145299152E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-CA89-4B9F-B6B5-36EEC4755D03}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1258327520"/>
+        <c:axId val="1258316000"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1258327520"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="fr-FR" sz="1400" b="0" i="1" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Deformation </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="el-GR" sz="1400" i="1">
+                    <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
+                  <a:t>ε</a:t>
+                </a:r>
+                <a:endParaRPr lang="fr-FR" sz="1400" b="0" i="1" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                </a:endParaRPr>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="fr-FR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1258316000"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1258316000"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="fr-FR" sz="1400" i="1">
+                    <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
+                  <a:t>ΔR/R0</a:t>
+                </a:r>
+                <a:endParaRPr lang="fr-FR" sz="1400" b="0" i="1" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                </a:endParaRPr>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="fr-FR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1258327520"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="9.3136701662292209E-2"/>
+          <c:y val="0.17171296296296296"/>
+          <c:w val="0.62421697287839017"/>
+          <c:h val="0.77736111111111106"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>5B Compression</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'5B compr'!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2.1099999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.3800000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.7100000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.1700000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.8E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.7499999999999999E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'5B compr'!$F$3:$F$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>-7.8586932115859588E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-1.0740214055834144E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-2.0657136441883092E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-2.7767382680937057E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-3.5008607140184118E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-4.9453633710051646E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-34ED-4BCD-BF47-0450E98CAF38}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1258335200"/>
+        <c:axId val="1258349120"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1258335200"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1258349120"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1258349120"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1258335200"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.74818000874890644"/>
+          <c:y val="0.46432742782152231"/>
+          <c:w val="0.23515332458442695"/>
+          <c:h val="0.22453922426363371"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>HB compression</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>HB Compression</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>('HB compr'!$C$3,'HB compr'!$C$4,'HB compr'!$C$6,'HB compr'!$C$8)</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2.1099999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.3800000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.1700000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.7499999999999999E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>('HB compr'!$F$3,'HB compr'!$F$4,'HB compr'!$F$6,'HB compr'!$F$8)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>-1.641025641025641E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-3.2324786324786324E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-3.433846153846154E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-6.2745299145299152E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C191-478A-88AC-930C9A0BC763}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1258352480"/>
+        <c:axId val="1258352960"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1258352480"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1258352960"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1258352960"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1258352480"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:legendEntry>
+        <c:idx val="2"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -1648,6 +3193,126 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2681,6 +4346,1554 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3207,9 +6420,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3299,6 +6512,129 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8399149E-DA6C-1B45-91BD-CFB47109EC97}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2150197</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>72767</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>356932</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>67901</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{344C776E-83D8-239D-A2B7-8F6239D5B015}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>335280</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>34290</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3ADD7596-63FF-3453-8020-108732AE30AB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>662940</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>163830</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>163830</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9896F0C-A3D4-FE4A-E07E-A6EA2286C6AF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3616,7 +6952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CF92F5E-7161-4D89-87DD-CF750AB5055C}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.77734375" bestFit="1" customWidth="1"/>
@@ -3624,153 +6960,177 @@
     <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2">
         <v>0</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>27209</v>
       </c>
-      <c r="D2">
-        <f>C2-$C$2</f>
+      <c r="E2">
+        <f>D2-$D$2</f>
         <v>0</v>
       </c>
-      <c r="E2">
-        <f>D2/$C$2</f>
+      <c r="F2">
+        <f>E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="C3">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.1099999999999999E-3</v>
+      </c>
+      <c r="D3">
         <v>27338</v>
       </c>
-      <c r="D3">
-        <f t="shared" ref="D3:D8" si="0">C3-$C$2</f>
+      <c r="E3">
+        <f>D3-$D$2</f>
         <v>129</v>
       </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E8" si="1">D3/$C$2</f>
+      <c r="F3">
+        <f>E3/$D$2</f>
         <v>4.7410783196736375E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>5.1000000000000004E-3</v>
-      </c>
-      <c r="C4">
+        <v>0.04</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.3800000000000002E-3</v>
+      </c>
+      <c r="D4">
         <v>27449</v>
       </c>
-      <c r="D4">
-        <f t="shared" si="0"/>
+      <c r="E4">
+        <f>D4-$D$2</f>
         <v>240</v>
       </c>
-      <c r="E4">
-        <f t="shared" si="1"/>
+      <c r="F4">
+        <f>E4/$D$2</f>
         <v>8.8206108272997907E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>6.3E-3</v>
-      </c>
-      <c r="C5">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2.7100000000000002E-3</v>
+      </c>
+      <c r="D5">
         <v>27894</v>
       </c>
-      <c r="D5">
-        <f t="shared" si="0"/>
+      <c r="E5">
+        <f>D5-$D$2</f>
         <v>685</v>
       </c>
-      <c r="E5">
-        <f t="shared" si="1"/>
+      <c r="F5">
+        <f>E5/$D$2</f>
         <v>2.517549340291815E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
-        <v>7.4999999999999997E-3</v>
+      <c r="B6">
+        <v>0.03</v>
       </c>
       <c r="C6" s="3">
+        <v>3.1700000000000001E-3</v>
+      </c>
+      <c r="D6">
         <v>28400</v>
       </c>
-      <c r="D6">
-        <f t="shared" si="0"/>
+      <c r="E6">
+        <f>D6-$D$2</f>
         <v>1191</v>
       </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
+      <c r="F6">
+        <f>E6/$D$2</f>
         <v>4.3772281230475212E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>8.6999999999999994E-3</v>
-      </c>
-      <c r="C7">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.8E-3</v>
+      </c>
+      <c r="D7">
         <v>28700</v>
       </c>
-      <c r="D7">
-        <f t="shared" si="0"/>
+      <c r="E7">
+        <f>D7-$D$2</f>
         <v>1491</v>
       </c>
-      <c r="E7">
-        <f t="shared" si="1"/>
+      <c r="F7">
+        <f>E7/$D$2</f>
         <v>5.479804476459995E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.01</v>
-      </c>
-      <c r="C8">
+        <v>0.02</v>
+      </c>
+      <c r="C8" s="3">
+        <v>4.7499999999999999E-3</v>
+      </c>
+      <c r="D8">
         <v>29050</v>
       </c>
-      <c r="D8">
-        <f t="shared" si="0"/>
+      <c r="E8">
+        <f>D8-$D$2</f>
         <v>1841</v>
       </c>
-      <c r="E8">
-        <f t="shared" si="1"/>
+      <c r="F8">
+        <f>E8/$D$2</f>
         <v>6.7661435554412147E-2</v>
       </c>
     </row>
@@ -3782,7 +7142,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C3BCE9-64D8-4C93-9C27-0CB4AD1314AB}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.77734375" bestFit="1" customWidth="1"/>
@@ -3790,153 +7150,177 @@
     <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>0</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>117000</v>
       </c>
-      <c r="D2">
-        <f>C2-$C$2</f>
+      <c r="E2">
+        <f>D2-$D$2</f>
         <v>0</v>
       </c>
-      <c r="E2">
-        <f>D2/$C$2</f>
+      <c r="F2">
+        <f>E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="C3">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.1099999999999999E-3</v>
+      </c>
+      <c r="D3">
         <v>123341</v>
       </c>
-      <c r="D3">
-        <f t="shared" ref="D3:D8" si="0">C3-$C$2</f>
+      <c r="E3">
+        <f>D3-$D$2</f>
         <v>6341</v>
       </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E8" si="1">D3/$C$2</f>
+      <c r="F3">
+        <f>E3/$D$2</f>
         <v>5.4196581196581196E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>5.1000000000000004E-3</v>
-      </c>
-      <c r="C4">
+        <v>0.04</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.3800000000000002E-3</v>
+      </c>
+      <c r="D4">
         <v>124672</v>
       </c>
-      <c r="D4">
-        <f t="shared" si="0"/>
+      <c r="E4">
+        <f>D4-$D$2</f>
         <v>7672</v>
       </c>
-      <c r="E4">
-        <f t="shared" si="1"/>
+      <c r="F4">
+        <f>E4/$D$2</f>
         <v>6.5572649572649577E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>6.3E-3</v>
-      </c>
-      <c r="C5">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2.7100000000000002E-3</v>
+      </c>
+      <c r="D5">
         <v>125678</v>
       </c>
-      <c r="D5">
-        <f t="shared" si="0"/>
+      <c r="E5">
+        <f>D5-$D$2</f>
         <v>8678</v>
       </c>
-      <c r="E5">
-        <f t="shared" si="1"/>
+      <c r="F5">
+        <f>E5/$D$2</f>
         <v>7.4170940170940169E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
-        <v>7.4999999999999997E-3</v>
-      </c>
-      <c r="C6">
+      <c r="B6">
+        <v>0.03</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3.1700000000000001E-3</v>
+      </c>
+      <c r="D6">
         <v>127400</v>
       </c>
-      <c r="D6">
-        <f t="shared" si="0"/>
+      <c r="E6">
+        <f>D6-$D$2</f>
         <v>10400</v>
       </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
+      <c r="F6">
+        <f>E6/$D$2</f>
         <v>8.8888888888888892E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>8.6999999999999994E-3</v>
-      </c>
-      <c r="C7">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.8E-3</v>
+      </c>
+      <c r="D7">
         <v>128096</v>
       </c>
-      <c r="D7">
-        <f t="shared" si="0"/>
+      <c r="E7">
+        <f>D7-$D$2</f>
         <v>11096</v>
       </c>
-      <c r="E7">
-        <f t="shared" si="1"/>
+      <c r="F7">
+        <f>E7/$D$2</f>
         <v>9.4837606837606836E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>0.01</v>
-      </c>
-      <c r="C8">
+        <v>0.02</v>
+      </c>
+      <c r="C8" s="3">
+        <v>4.7499999999999999E-3</v>
+      </c>
+      <c r="D8">
         <v>132320</v>
       </c>
-      <c r="D8">
-        <f t="shared" si="0"/>
+      <c r="E8">
+        <f>D8-$D$2</f>
         <v>15320</v>
       </c>
-      <c r="E8">
-        <f t="shared" si="1"/>
+      <c r="F8">
+        <f>E8/$D$2</f>
         <v>0.13094017094017094</v>
       </c>
     </row>
@@ -3948,7 +7332,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCF125B-5851-4C8E-A3AF-C4DCB05BA689}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.77734375" bestFit="1" customWidth="1"/>
@@ -3956,135 +7340,720 @@
     <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>0</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>186800</v>
       </c>
-      <c r="D2">
-        <f>C2-$C$2</f>
+      <c r="E2">
+        <f>D2-$D$2</f>
         <v>0</v>
       </c>
-      <c r="E2">
-        <f>D2/$C$2</f>
+      <c r="F2">
+        <f>E2/$D$2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="C3">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.1099999999999999E-3</v>
+      </c>
+      <c r="D3">
         <v>210600</v>
       </c>
-      <c r="D3">
-        <f t="shared" ref="D3:D7" si="0">C3-$C$2</f>
+      <c r="E3">
+        <f>D3-$D$2</f>
         <v>23800</v>
       </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E7" si="1">D3/$C$2</f>
+      <c r="F3">
+        <f>E3/$D$2</f>
         <v>0.12740899357601712</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>6.3E-3</v>
-      </c>
-      <c r="C4">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.7100000000000002E-3</v>
+      </c>
+      <c r="D4">
         <v>214560</v>
       </c>
-      <c r="D4">
-        <f t="shared" si="0"/>
+      <c r="E4">
+        <f>D4-$D$2</f>
         <v>27760</v>
       </c>
-      <c r="E4">
-        <f t="shared" si="1"/>
+      <c r="F4">
+        <f>E4/$D$2</f>
         <v>0.14860813704496789</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>7.4999999999999997E-3</v>
-      </c>
-      <c r="C5">
+        <v>0.03</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.1700000000000001E-3</v>
+      </c>
+      <c r="D5">
         <v>219000</v>
       </c>
-      <c r="D5">
-        <f t="shared" si="0"/>
+      <c r="E5">
+        <f>D5-$D$2</f>
         <v>32200</v>
       </c>
-      <c r="E5">
-        <f t="shared" si="1"/>
+      <c r="F5">
+        <f>E5/$D$2</f>
         <v>0.17237687366167023</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>8.6999999999999994E-3</v>
-      </c>
-      <c r="C6">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3.8E-3</v>
+      </c>
+      <c r="D6">
         <v>223736</v>
       </c>
-      <c r="D6">
-        <f t="shared" si="0"/>
+      <c r="E6">
+        <f>D6-$D$2</f>
         <v>36936</v>
       </c>
-      <c r="E6">
-        <f t="shared" si="1"/>
+      <c r="F6">
+        <f>E6/$D$2</f>
         <v>0.19773019271948608</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>0.01</v>
-      </c>
-      <c r="C7" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="C7" s="3">
+        <v>4.7499999999999999E-3</v>
+      </c>
+      <c r="D7" s="1">
         <v>234560</v>
       </c>
+      <c r="E7">
+        <f>D7-$D$2</f>
+        <v>47760</v>
+      </c>
+      <c r="F7">
+        <f>E7/$D$2</f>
+        <v>0.25567451820128478</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBE14704-9C8A-4370-B3B7-9AB02F7FD6E1}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>48578</v>
+      </c>
+      <c r="E2">
+        <f>D2-$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <f>E2/$D$2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>-4.4999999999999998E-2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.1099999999999999E-3</v>
+      </c>
+      <c r="D3">
+        <v>48006</v>
+      </c>
+      <c r="E3">
+        <f>D3-$D$2</f>
+        <v>-572</v>
+      </c>
+      <c r="F3">
+        <f>E3/$D$2</f>
+        <v>-1.1774877516571287E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>-0.04</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.3800000000000002E-3</v>
+      </c>
+      <c r="D4">
+        <v>47970</v>
+      </c>
+      <c r="E4">
+        <f>D4-$D$2</f>
+        <v>-608</v>
+      </c>
+      <c r="F4">
+        <f>E4/$D$2</f>
+        <v>-1.2515953723907942E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>-3.5000000000000003E-2</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.7100000000000002E-3</v>
+      </c>
+      <c r="D5" s="4">
+        <v>47269</v>
+      </c>
+      <c r="E5" s="4">
+        <f>D5-$D$2</f>
+        <v>-1309</v>
+      </c>
+      <c r="F5" s="4">
+        <f>E5/$D$2</f>
+        <v>-2.6946354316768908E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>-0.03</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3.1700000000000001E-3</v>
+      </c>
+      <c r="D6">
+        <v>47400</v>
+      </c>
+      <c r="E6">
+        <f>D6-$D$2</f>
+        <v>-1178</v>
+      </c>
+      <c r="F6">
+        <f>E6/$D$2</f>
+        <v>-2.4249660340071637E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>-2.5000000000000001E-2</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.8E-3</v>
+      </c>
       <c r="D7">
-        <f t="shared" si="0"/>
-        <v>47760</v>
+        <v>47115</v>
       </c>
       <c r="E7">
-        <f t="shared" si="1"/>
-        <v>0.25567451820128478</v>
+        <f>D7-$D$2</f>
+        <v>-1463</v>
+      </c>
+      <c r="F7">
+        <f>E7/$D$2</f>
+        <v>-3.0116513648153487E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-0.02</v>
+      </c>
+      <c r="C8" s="5">
+        <v>4.7499999999999999E-3</v>
+      </c>
+      <c r="D8" s="4">
+        <v>48387</v>
+      </c>
+      <c r="E8" s="4">
+        <f>D8-$D$2</f>
+        <v>-191</v>
+      </c>
+      <c r="F8" s="4">
+        <f>E8/$D$2</f>
+        <v>-3.9318209889250277E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F1D1FAB-936E-4C77-8731-F3F5C599C03B}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>53444</v>
+      </c>
+      <c r="E2">
+        <f>D2-$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <f>E2/$D$2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.1099999999999999E-3</v>
+      </c>
+      <c r="D3">
+        <v>53024</v>
+      </c>
+      <c r="E3">
+        <f>D3-$D$2</f>
+        <v>-420</v>
+      </c>
+      <c r="F3">
+        <f>E3/$D$2</f>
+        <v>-7.8586932115859588E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0.04</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.3800000000000002E-3</v>
+      </c>
+      <c r="D4">
+        <v>52870</v>
+      </c>
+      <c r="E4">
+        <f>D4-$D$2</f>
+        <v>-574</v>
+      </c>
+      <c r="F4">
+        <f>E4/$D$2</f>
+        <v>-1.0740214055834144E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2.7100000000000002E-3</v>
+      </c>
+      <c r="D5">
+        <v>52340</v>
+      </c>
+      <c r="E5">
+        <f>D5-$D$2</f>
+        <v>-1104</v>
+      </c>
+      <c r="F5">
+        <f>E5/$D$2</f>
+        <v>-2.0657136441883092E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0.03</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3.1700000000000001E-3</v>
+      </c>
+      <c r="D6">
+        <v>51960</v>
+      </c>
+      <c r="E6">
+        <f>D6-$D$2</f>
+        <v>-1484</v>
+      </c>
+      <c r="F6">
+        <f>E6/$D$2</f>
+        <v>-2.7767382680937057E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.8E-3</v>
+      </c>
+      <c r="D7">
+        <v>51573</v>
+      </c>
+      <c r="E7">
+        <f>D7-$D$2</f>
+        <v>-1871</v>
+      </c>
+      <c r="F7">
+        <f>E7/$D$2</f>
+        <v>-3.5008607140184118E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>0.02</v>
+      </c>
+      <c r="C8" s="3">
+        <v>4.7499999999999999E-3</v>
+      </c>
+      <c r="D8">
+        <v>50801</v>
+      </c>
+      <c r="E8">
+        <f>D8-$D$2</f>
+        <v>-2643</v>
+      </c>
+      <c r="F8">
+        <f>E8/$D$2</f>
+        <v>-4.9453633710051646E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C954F671-BD54-4778-A3FA-5038C1C49DF3}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>585000</v>
+      </c>
+      <c r="E2">
+        <f>D2-$D$2</f>
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <f>E2/$D$2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.1099999999999999E-3</v>
+      </c>
+      <c r="D3">
+        <v>575400</v>
+      </c>
+      <c r="E3">
+        <f>D3-$D$2</f>
+        <v>-9600</v>
+      </c>
+      <c r="F3">
+        <f>E3/$D$2</f>
+        <v>-1.641025641025641E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0.04</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.3800000000000002E-3</v>
+      </c>
+      <c r="D4">
+        <v>566090</v>
+      </c>
+      <c r="E4">
+        <f>D4-$D$2</f>
+        <v>-18910</v>
+      </c>
+      <c r="F4">
+        <f>E4/$D$2</f>
+        <v>-3.2324786324786324E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2.7100000000000002E-3</v>
+      </c>
+      <c r="D5" s="4">
+        <v>565408</v>
+      </c>
+      <c r="E5" s="4">
+        <f>D5-$D$2</f>
+        <v>-19592</v>
+      </c>
+      <c r="F5" s="4">
+        <f>E5/$D$2</f>
+        <v>-3.3490598290598292E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0.03</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3.1700000000000001E-3</v>
+      </c>
+      <c r="D6">
+        <v>564912</v>
+      </c>
+      <c r="E6">
+        <f>D6-$D$2</f>
+        <v>-20088</v>
+      </c>
+      <c r="F6">
+        <f>E6/$D$2</f>
+        <v>-3.433846153846154E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="6">
+        <v>5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="C7" s="5">
+        <v>3.8E-3</v>
+      </c>
+      <c r="D7" s="6">
+        <v>561021</v>
+      </c>
+      <c r="E7" s="4">
+        <f>D7-$D$2</f>
+        <v>-23979</v>
+      </c>
+      <c r="F7" s="4">
+        <f>E7/$D$2</f>
+        <v>-4.0989743589743589E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>0.02</v>
+      </c>
+      <c r="C8" s="3">
+        <v>4.7499999999999999E-3</v>
+      </c>
+      <c r="D8">
+        <v>548294</v>
+      </c>
+      <c r="E8">
+        <f>D8-$D$2</f>
+        <v>-36706</v>
+      </c>
+      <c r="F8">
+        <f>E8/$D$2</f>
+        <v>-6.2745299145299152E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>